<commit_message>
Add QA report PRISM_Report_2026-06-11.xlsx
</commit_message>
<xml_diff>
--- a/reports/PRISM_Report_2026-06-11.xlsx
+++ b/reports/PRISM_Report_2026-06-11.xlsx
@@ -403,10 +403,10 @@
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="50.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -432,7 +432,7 @@
         <v>Video 3</v>
       </c>
       <c r="H1" t="str">
-        <v>Summary</v>
+        <v>comments</v>
       </c>
     </row>
     <row r="2">
@@ -510,7 +510,7 @@
         <v>—</v>
       </c>
       <c r="H4" t="str">
-        <v>Video 1 has no passing metrics</v>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -536,7 +536,7 @@
         <v>—</v>
       </c>
       <c r="H5" t="str">
-        <v>Video 2 has no passing metrics</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -692,7 +692,7 @@
         <v>Yes</v>
       </c>
       <c r="H11" t="str">
-        <v>Video 1 has Brightness, Noise: Slight, Avg, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -718,7 +718,7 @@
         <v>Yes</v>
       </c>
       <c r="H12" t="str">
-        <v>Video 2 has Brightness, Noise, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -744,7 +744,7 @@
         <v>Yes</v>
       </c>
       <c r="H13" t="str">
-        <v>Video 3 has Wobble, Jitter, Brightness, Noise, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -874,7 +874,7 @@
         <v>Yes</v>
       </c>
       <c r="H18" t="str">
-        <v>Video 1 has Jitter, Noise</v>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -900,7 +900,7 @@
         <v>Yes</v>
       </c>
       <c r="H19" t="str">
-        <v>Video 2 has Wobble, Jitter, Brightness, Noise, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -926,7 +926,7 @@
         <v>Yes</v>
       </c>
       <c r="H20" t="str">
-        <v>Video 3 has Wobble, Jitter, Brightness, Noise, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1056,7 +1056,7 @@
         <v>Yes</v>
       </c>
       <c r="H25" t="str">
-        <v>Video 1 has Brightness, Noise: Slight, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1082,7 +1082,7 @@
         <v>Yes</v>
       </c>
       <c r="H26" t="str">
-        <v>Video 2 has Brightness, Noise, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1108,7 +1108,7 @@
         <v>Yes</v>
       </c>
       <c r="H27" t="str">
-        <v>Video 3 has Wobble, Jitter, Brightness, Noise, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1238,7 +1238,7 @@
         <v>—</v>
       </c>
       <c r="H32" t="str">
-        <v>Video 1 has Brightness, Noise: Slight, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -1264,7 +1264,7 @@
         <v>—</v>
       </c>
       <c r="H33" t="str">
-        <v>Video 2 has Brightness, Noise, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -1420,7 +1420,7 @@
         <v>Yes</v>
       </c>
       <c r="H39" t="str">
-        <v>Video 1 has Brightness, Noise: Slight, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -1446,7 +1446,7 @@
         <v>Yes</v>
       </c>
       <c r="H40" t="str">
-        <v>Video 2 has Brightness, Noise, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -1472,7 +1472,7 @@
         <v>Yes</v>
       </c>
       <c r="H41" t="str">
-        <v>Video 3 has Wobble, Jitter, Brightness, Noise, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -1602,7 +1602,7 @@
         <v>Yes</v>
       </c>
       <c r="H46" t="str">
-        <v>Video 1 has Jitter: Not good, Brightness, Noise: Slight, Stability</v>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -1619,16 +1619,16 @@
         <v>Jitter</v>
       </c>
       <c r="E47" t="str">
-        <v>No (Not good)</v>
+        <v>No</v>
       </c>
       <c r="F47" t="str">
         <v>No</v>
       </c>
       <c r="G47" t="str">
-        <v>Yes (Excellent)</v>
+        <v>Yes</v>
       </c>
       <c r="H47" t="str">
-        <v>Video 2 has Brightness (very good), Noise, Stability</v>
+        <v>Video 3: Very good</v>
       </c>
     </row>
     <row r="48">
@@ -1645,16 +1645,16 @@
         <v>Brightness</v>
       </c>
       <c r="E48" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="F48" t="str">
-        <v>Yes (very good)</v>
+        <v>Yes</v>
       </c>
       <c r="G48" t="str">
         <v>Yes</v>
       </c>
       <c r="H48" t="str">
-        <v>Video 3 has Wobble, Jitter (Excellent), Brightness, Noise, Stability</v>
+        <v>Video 1: not real, Video 2: Real</v>
       </c>
     </row>
     <row r="49">

</xml_diff>